<commit_message>
Add Ribo-seq ORF catalogues for zebrafish, C. elegans and yeast, and optional human ones
Yang et al.'s RibORF 2.0 ORFs (Nat Commun 2024) for each species:
riborf-zebrafish (9,759 on GRCz11, Ensembl 115), riborf-worm (2,849 on
WBcel235, Ensembl 105) and riborf-yeast (1,124 on R64-1-1, placed from
genomic spans because the source's yeast transcripts carry UTRs that
Ensembl's lack). Human gets Chang et al.'s ncORFs (11,621) and Yang et
al.'s ORFs (51,174) as optional catalogues: the bundled GENCODE set
stays human's offline default, and catalogs="all" (load_catalog,
extra_orfs, Proteome.build, install_species, --catalogs) adds them.

The RibORF importer keeps C. elegans names with dots whole and leaves
ORFs over ambiguous bases unresolved; the mouse catalogue it builds is
byte-identical to 0.28.0's. Docs record that no public dog Ribo-seq or
ncORF MS search exists. Version 0.29.0.

Claude-Session: https://claude.ai/code/session_016N35AjLGwyYtEcjeN5k6mT
</commit_message>
<xml_diff>
--- a/tests/data/ncorf_mammals/S3.xlsx
+++ b/tests/data/ncorf_mammals/S3.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,6 +919,293 @@
       </c>
       <c r="S7" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1_167936685_167936702_+</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>uORF</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ATG</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>167936685</v>
+      </c>
+      <c r="I8" t="n">
+        <v>167936702</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ENSG00000143164</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>protein_coding</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>ENST00000367840</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>20</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1_53838293_53838276_-</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>uORF</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CTG</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>53838293</v>
+      </c>
+      <c r="I9" t="n">
+        <v>53838276</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>ENSG00000058804</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>protein_coding</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>ENST00000371429</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="n">
+        <v>21</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>c1riboseqorf101</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>phase1</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>7_96709845_96709825_-</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>uORF</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GTG</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>96709845</v>
+      </c>
+      <c r="I10" t="n">
+        <v>96709825</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ENSG00000127922</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>protein_coding</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>ENST00000248566</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>22</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6_134530858_134525331_-</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>lncORF</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>234</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ATG</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>134530858</v>
+      </c>
+      <c r="I11" t="n">
+        <v>134525331</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ENSG00000232310</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>lncRNA</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ENST00000607531</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>817</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1050</v>
+      </c>
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Ribo-seq ORF catalogues for zebrafish, C. elegans and yeast, and optional human ones (#100)
Yang et al.'s RibORF 2.0 ORFs for zebrafish (9,759), C. elegans (2,849)
and yeast (1,128, placed from genomic spans), and Chang et al.'s and Yang
et al.'s human ORFs (11,621 and 51,174) as optional catalogues selected
with catalogs="all". The bundled GENCODE set stays human's default.

Claude-Session: https://claude.ai/code/session_016N35AjLGwyYtEcjeN5k6mT
</commit_message>
<xml_diff>
--- a/tests/data/ncorf_mammals/S3.xlsx
+++ b/tests/data/ncorf_mammals/S3.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,6 +919,293 @@
       </c>
       <c r="S7" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1_167936685_167936702_+</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>uORF</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ATG</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>167936685</v>
+      </c>
+      <c r="I8" t="n">
+        <v>167936702</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ENSG00000143164</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>protein_coding</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>ENST00000367840</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>20</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1_53838293_53838276_-</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>uORF</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CTG</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>53838293</v>
+      </c>
+      <c r="I9" t="n">
+        <v>53838276</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>ENSG00000058804</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>protein_coding</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>ENST00000371429</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="n">
+        <v>21</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>c1riboseqorf101</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>phase1</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>7_96709845_96709825_-</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>uORF</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GTG</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>96709845</v>
+      </c>
+      <c r="I10" t="n">
+        <v>96709825</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ENSG00000127922</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>protein_coding</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>ENST00000248566</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>22</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6_134530858_134525331_-</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>lncORF</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>234</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ATG</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>134530858</v>
+      </c>
+      <c r="I11" t="n">
+        <v>134525331</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ENSG00000232310</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>lncRNA</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ENST00000607531</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>817</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1050</v>
+      </c>
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>